<commit_message>
Complete smooth circuit: replace Uluwatu with Sanur beachfront villa in Atlas and budget ledger
</commit_message>
<xml_diff>
--- a/Bali Sanctuary Смета 4 звезды.xlsx
+++ b/Bali Sanctuary Смета 4 звезды.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="539">
   <si>
     <t>СРАВНИТЕЛЬНАЯ СМЕТА: ИСХОДНАЯ СМЕТА (МАРАТ 5★) vs АКТУАЛЬНАЯ (ШВЕЙЦАРИЯ 4★+)</t>
   </si>
@@ -36,345 +36,348 @@
     <t>Актуально (Швейцария, 4★) [€]</t>
   </si>
   <si>
+    <t>Стоимость in IDR</t>
+  </si>
+  <si>
+    <t>Разница / Экономия [€]</t>
+  </si>
+  <si>
+    <t>Официальный источник / Ссылка</t>
+  </si>
+  <si>
+    <t>1. Размещение</t>
+  </si>
+  <si>
+    <t>Убуд: Plataran Ubud Hotel &amp; Spa (Deluxe Suite, 320 €/н) vs The Kayon Jungle (850 €/н)</t>
+  </si>
+  <si>
+    <t>3 ночи</t>
+  </si>
+  <si>
+    <t>-1 590 € (экономия)</t>
+  </si>
+  <si>
+    <t>plataran.com/plataran-ubud</t>
+  </si>
+  <si>
+    <t>Кинтамани: Toteme Glamping &amp; Hot Springs (Шатер с купелью, 220 €) vs Faro Cabin (350 €)</t>
+  </si>
+  <si>
+    <t>1 ночь</t>
+  </si>
+  <si>
+    <t>-130 € (экономия)</t>
+  </si>
+  <si>
+    <t>totemeglamping.com</t>
+  </si>
+  <si>
+    <t>Побережье: Приватная вилла у пляжа (Paradise Beach / Санур, 340 €/н) vs Bulgari / Six Senses (1 000 €/н)</t>
+  </si>
+  <si>
+    <t>2 ночи</t>
+  </si>
+  <si>
+    <t>-1 320 € (экономия)</t>
+  </si>
+  <si>
+    <t>Приватная бутик-вилла на первой линии</t>
+  </si>
+  <si>
+    <t>ИТОГО ПРОЖИВАНИЕ (6 ночей, средняя 310 €/ночь против 815 €/ночь)</t>
+  </si>
+  <si>
+    <t>6 ночей</t>
+  </si>
+  <si>
+    <t>-3 040 € (экономия)</t>
+  </si>
+  <si>
+    <t>Экономия перенаправлена в маржу</t>
+  </si>
+  <si>
+    <t>2. Логистика и авто</t>
+  </si>
+  <si>
+    <t>Личный водитель Путу &amp; Toyota Innova Zenix 24/7 (с бензином и ожиданием)</t>
+  </si>
+  <si>
+    <t>7 дней</t>
+  </si>
+  <si>
+    <t>-110 € (выгодный тариф)</t>
+  </si>
+  <si>
+    <t>1 100 000 IDR/день (Путу WhatsApp)</t>
+  </si>
+  <si>
+    <t>Встречи/проводы, ночные переезды, парковки, платные хайвеи Bali Mandara</t>
+  </si>
+  <si>
+    <t>+10 €</t>
+  </si>
+  <si>
+    <t>Фактические дорожные сборы</t>
+  </si>
+  <si>
+    <t>ИТОГО ТРАНСПОРТ И ПУТУ НА ВЕСЬ МАРШРУТ</t>
+  </si>
+  <si>
+    <t>-100 € (экономия)</t>
+  </si>
+  <si>
+    <t>100% готовность и безопасность</t>
+  </si>
+  <si>
+    <t>3. VIP Аэропорт и въезд</t>
+  </si>
+  <si>
+    <t>VIP Fast-Track (JOUMPA Garuda): Meet &amp; Greet у трапа, дип-коридор, портье багажа, VIP Lounge</t>
+  </si>
+  <si>
+    <t>2 чел</t>
+  </si>
+  <si>
+    <t>+110 € (полный VIP)</t>
+  </si>
+  <si>
+    <t>joumpa.com (80 €/чел за полный VIP)</t>
+  </si>
+  <si>
+    <t>Электронная виза e-VOA B1 (официальный портал Иммиграции)</t>
+  </si>
+  <si>
+    <t>+4 € (курс)</t>
+  </si>
+  <si>
+    <t>evisa.imigrasi.go.id (500 000 IDR/чел)</t>
+  </si>
+  <si>
+    <t>Официальный туристический сбор Бали (Love Bali Tourist Levy)</t>
+  </si>
+  <si>
+    <t>0 €</t>
+  </si>
+  <si>
+    <t>lovebali.baliprov.go.id (150 000 IDR/чел)</t>
+  </si>
+  <si>
+    <t>ИТОГО ВЪЕЗДНЫЕ СБОРЫ И VIP ПРИЛЕТ (ВКЛЮЧАЯ ПОРТЬЕ И ЛАУНЖ)</t>
+  </si>
+  <si>
+    <t>+114 € (премиум комфорт)</t>
+  </si>
+  <si>
+    <t>Оформляется организатором заранее</t>
+  </si>
+  <si>
+    <t>4. Спа и релаксация</t>
+  </si>
+  <si>
+    <t>3-часовой ритуал: ванна из роз, скраб Lulur, травяной уход (Padma Spa Plataran)</t>
+  </si>
+  <si>
+    <t>-10 €</t>
+  </si>
+  <si>
+    <t>Фирменный спа Plataran</t>
+  </si>
+  <si>
+    <t>Восстанавливающие балийские массажи и релакс-терапия</t>
+  </si>
+  <si>
+    <t>2 чел х 2 раза</t>
+  </si>
+  <si>
+    <t>+50 €</t>
+  </si>
+  <si>
+    <t>Сертифицированные мастера</t>
+  </si>
+  <si>
+    <t>ИТОГО СПА-ПРОГРАММА</t>
+  </si>
+  <si>
+    <t>Комплекс</t>
+  </si>
+  <si>
+    <t>+40 €</t>
+  </si>
+  <si>
+    <t>Глубокая телесная перезагрузка</t>
+  </si>
+  <si>
+    <t>5. Места Силы &amp; Обряды</t>
+  </si>
+  <si>
+    <t>Церемония Мелукат у священника Манку + подношения (каньон Себату)</t>
+  </si>
+  <si>
+    <t>-15 €</t>
+  </si>
+  <si>
+    <t>Скрытый водопад Genah Melukat</t>
+  </si>
+  <si>
+    <t>Агни-хотра (огненная ведическая пуджа) с потомственным священником</t>
+  </si>
+  <si>
+    <t>Сессия</t>
+  </si>
+  <si>
+    <t>+20 €</t>
+  </si>
+  <si>
+    <t>Индивидуальный сакральный обряд</t>
+  </si>
+  <si>
+    <t>Билеты в храмы: Бесаких, Батукару, Себату, термы Батур, Ботанический сад</t>
+  </si>
+  <si>
+    <t>Входные билеты, саронги, шаттлы</t>
+  </si>
+  <si>
+    <t>ИТОГО САКРАЛЬНАЯ ПРОГРАММА</t>
+  </si>
+  <si>
+    <t>+15 €</t>
+  </si>
+  <si>
+    <t>Закрытый доступ без толп туристов</t>
+  </si>
+  <si>
+    <t>6. Гастрономия</t>
+  </si>
+  <si>
+    <t>Приветственный ужин на вилле + тропические фрукты ежедневно (мангостины, маракуйя)</t>
+  </si>
+  <si>
+    <t>Ежедневная свежая экзотика</t>
+  </si>
+  <si>
+    <t>Авторский дегустационный сет от шефа (Mozaic / Locavore NXT)</t>
+  </si>
+  <si>
+    <t>Гастрономический флагман Азии</t>
+  </si>
+  <si>
+    <t>Праздничный закатный ужин морепродуктов на берегу океана (Санур)</t>
+  </si>
+  <si>
+    <t>Свежий улов дня у самой воды</t>
+  </si>
+  <si>
+    <t>ИТОГО ПИТАНИЕ И НАПИТКИ</t>
+  </si>
+  <si>
+    <t>Отобранные шеф-локации</t>
+  </si>
+  <si>
+    <t>7. Проводник &amp; Арт</t>
+  </si>
+  <si>
+    <t>Звукотерапия тибетскими чашами от Валерия на вилле (2 сессии)</t>
+  </si>
+  <si>
+    <t>2 сессии</t>
+  </si>
+  <si>
+    <t>Включено</t>
+  </si>
+  <si>
+    <t>Авторская практика мастера</t>
+  </si>
+  <si>
+    <t>Авторская fine-art портретная фотосъемка на закатном побережье</t>
+  </si>
+  <si>
+    <t>1 сессия</t>
+  </si>
+  <si>
+    <t>Fine-art фотосессия для гостий от Валерия</t>
+  </si>
+  <si>
+    <t>Интеллектуальный салон: встреча с д-ром Лоуренсом Блэром («Ring of Fire»)</t>
+  </si>
+  <si>
+    <t>1 встреча</t>
+  </si>
+  <si>
+    <t>Эксклюзивный доступ автора (35 лет экспедиций)</t>
+  </si>
+  <si>
+    <t>Частный визит в резиденцию Брюса Карпентера (сакральные крисы и маски)</t>
+  </si>
+  <si>
+    <t>1 визит</t>
+  </si>
+  <si>
+    <t>Эксперт Christie's / автор монографий</t>
+  </si>
+  <si>
+    <t>Арт-маршрут Убуда: музей Бланко, Neka Art Museum (павильон крисов), ARMA</t>
+  </si>
+  <si>
+    <t>1 день</t>
+  </si>
+  <si>
+    <t>Билеты включены в общую сакральную программу</t>
+  </si>
+  <si>
+    <t>Непрерывное кураторство 24/7 (индонезийский и английский языки)</t>
+  </si>
+  <si>
+    <t>Личное ведение без посредников</t>
+  </si>
+  <si>
+    <t>ИТОГО ОПЕРАЦИОННАЯ СЕБЕСТОИМОСТЬ (40%)</t>
+  </si>
+  <si>
+    <t>Прямые расходы на 2 гостей (отели 4★+, авто, спа, храмы, еда, VIP)</t>
+  </si>
+  <si>
+    <t>-2 388 € (чистая экономия)</t>
+  </si>
+  <si>
+    <t>40% от общей суммы пакета</t>
+  </si>
+  <si>
+    <t>ГОНОРАР МАСТЕРА ВАЛЕРИЯ ЛАТЫПОВА (60%)</t>
+  </si>
+  <si>
+    <t>Чистый гонорар за организацию, режиссуру тура и личное ведение</t>
+  </si>
+  <si>
+    <t>+4 688 € (рост гонорара)</t>
+  </si>
+  <si>
+    <t>60% чистая маржа автора</t>
+  </si>
+  <si>
+    <t>ИТОГОВАЯ СТОИМОСТЬ ПАКЕТА (ДЛЯ 2 ГОСТЕЙ)</t>
+  </si>
+  <si>
+    <t>Полный пакет «под ключ» (без международных авиабилетов)</t>
+  </si>
+  <si>
+    <t>+2 300 € (премиум Швейцария)</t>
+  </si>
+  <si>
+    <t>12 000 € за тур на двоих</t>
+  </si>
+  <si>
+    <t>СМЕТА ТУРА «BALI SANCTUARY»: 5 ДНЕЙ / 4 НОЧИ (ГОСТЬИ ИЗ ШВЕЙЦАРИИ)</t>
+  </si>
+  <si>
+    <t>Камерные бутик-отели 4★+ (300–400 €/ночь) • Полный VIP Fast-Track • Гонорар мастера 60%</t>
+  </si>
+  <si>
+    <t>Базовый расчет 5★ [€]</t>
+  </si>
+  <si>
     <t>Стоимость в IDR</t>
   </si>
   <si>
-    <t>Разница / Экономия [€]</t>
-  </si>
-  <si>
-    <t>Официальный источник / Ссылка</t>
-  </si>
-  <si>
-    <t>1. Размещение</t>
-  </si>
-  <si>
-    <t>Убуд: Plataran Ubud Hotel &amp; Spa (Deluxe Suite, 320 €/н) vs The Kayon Jungle (850 €/н)</t>
-  </si>
-  <si>
-    <t>3 ночи</t>
-  </si>
-  <si>
-    <t>-1 590 € (экономия)</t>
-  </si>
-  <si>
-    <t>plataran.com/plataran-ubud</t>
-  </si>
-  <si>
-    <t>Кинтамани: Toteme Glamping &amp; Hot Springs (Шатер с купелью, 220 €) vs Faro Cabin (350 €)</t>
-  </si>
-  <si>
-    <t>1 ночь</t>
-  </si>
-  <si>
-    <t>-130 € (экономия)</t>
-  </si>
-  <si>
-    <t>totemeglamping.com</t>
-  </si>
-  <si>
-    <t>Улувату: Renaissance Uluwatu (Ocean Suite, 340 €/н) vs Bulgari / Six Senses (1 000 €/н)</t>
-  </si>
-  <si>
-    <t>2 ночи</t>
-  </si>
-  <si>
-    <t>-1 320 € (экономия)</t>
-  </si>
-  <si>
-    <t>marriott.com/renaissance-bali</t>
-  </si>
-  <si>
-    <t>ИТОГО ПРОЖИВАНИЕ (6 ночей, средняя 310 €/ночь против 815 €/ночь)</t>
-  </si>
-  <si>
-    <t>6 ночей</t>
-  </si>
-  <si>
-    <t>-3 040 € (экономия)</t>
-  </si>
-  <si>
-    <t>Экономия перенаправлена в маржу</t>
-  </si>
-  <si>
-    <t>2. Логистика и авто</t>
-  </si>
-  <si>
-    <t>Личный водитель Путу &amp; Toyota Innova Zenix 24/7 (с бензином и ожиданием)</t>
-  </si>
-  <si>
-    <t>7 дней</t>
-  </si>
-  <si>
-    <t>-110 € (выгодный тариф)</t>
-  </si>
-  <si>
-    <t>1 100 000 IDR/день (Путу WhatsApp)</t>
-  </si>
-  <si>
-    <t>Встречи/проводы, ночные переезды, парковки, платные хайвеи Bali Mandara</t>
-  </si>
-  <si>
-    <t>+10 €</t>
-  </si>
-  <si>
-    <t>Фактические дорожные сборы</t>
-  </si>
-  <si>
-    <t>ИТОГО ТРАНСПОРТ И ПУТУ НА ВЕСЬ МАРШРУТ</t>
-  </si>
-  <si>
-    <t>-100 € (экономия)</t>
-  </si>
-  <si>
-    <t>100% готовность и безопасность</t>
-  </si>
-  <si>
-    <t>3. VIP Аэропорт и въезд</t>
-  </si>
-  <si>
-    <t>VIP Fast-Track (JOUMPA Garuda): Meet &amp; Greet у трапа, дип-коридор, портье багажа, VIP Lounge</t>
-  </si>
-  <si>
-    <t>2 чел</t>
-  </si>
-  <si>
-    <t>+110 € (полный VIP)</t>
-  </si>
-  <si>
-    <t>joumpa.com (80 €/чел за полный VIP)</t>
-  </si>
-  <si>
-    <t>Электронная виза e-VOA B1 (официальный портал Иммиграции)</t>
-  </si>
-  <si>
-    <t>+4 € (курс)</t>
-  </si>
-  <si>
-    <t>evisa.imigrasi.go.id (500 000 IDR/чел)</t>
-  </si>
-  <si>
-    <t>Официальный туристический сбор Бали (Love Bali Tourist Levy)</t>
-  </si>
-  <si>
-    <t>0 €</t>
-  </si>
-  <si>
-    <t>lovebali.baliprov.go.id (150 000 IDR/чел)</t>
-  </si>
-  <si>
-    <t>ИТОГО ВЪЕЗДНЫЕ СБОРЫ И VIP ПРИЛЕТ (ВКЛЮЧАЯ ПОРТЬЕ И ЛАУНЖ)</t>
-  </si>
-  <si>
-    <t>+114 € (премиум комфорт)</t>
-  </si>
-  <si>
-    <t>Оформляется организатором заранее</t>
-  </si>
-  <si>
-    <t>4. Спа и релаксация</t>
-  </si>
-  <si>
-    <t>3-часовой ритуал: ванна из роз, скраб Lulur, травяной уход (Padma Spa Plataran)</t>
-  </si>
-  <si>
-    <t>-10 €</t>
-  </si>
-  <si>
-    <t>Фирменный спа Plataran</t>
-  </si>
-  <si>
-    <t>Восстанавливающие балийские массажи и релакс-терапия</t>
-  </si>
-  <si>
-    <t>2 чел х 2 раза</t>
-  </si>
-  <si>
-    <t>+50 €</t>
-  </si>
-  <si>
-    <t>Сертифицированные мастера</t>
-  </si>
-  <si>
-    <t>ИТОГО СПА-ПРОГРАММА</t>
-  </si>
-  <si>
-    <t>Комплекс</t>
-  </si>
-  <si>
-    <t>+40 €</t>
-  </si>
-  <si>
-    <t>Глубокая телесная перезагрузка</t>
-  </si>
-  <si>
-    <t>5. Места Силы &amp; Обряды</t>
-  </si>
-  <si>
-    <t>Церемония Мелукат у священника Манку + подношения (каньон Себату)</t>
-  </si>
-  <si>
-    <t>-15 €</t>
-  </si>
-  <si>
-    <t>Скрытый водопад Genah Melukat</t>
-  </si>
-  <si>
-    <t>Агни-хотра (огненная ведическая пуджа) с потомственным священником</t>
-  </si>
-  <si>
-    <t>Сессия</t>
-  </si>
-  <si>
-    <t>+20 €</t>
-  </si>
-  <si>
-    <t>Индивидуальный сакральный обряд</t>
-  </si>
-  <si>
-    <t>Билеты в храмы: Бесаких, Батукару, Себату, термы Батур, Ботанический сад</t>
-  </si>
-  <si>
-    <t>Входные билеты, саронги, шаттлы</t>
-  </si>
-  <si>
-    <t>ИТОГО САКРАЛЬНАЯ ПРОГРАММА</t>
-  </si>
-  <si>
-    <t>+15 €</t>
-  </si>
-  <si>
-    <t>Закрытый доступ без толп туристов</t>
-  </si>
-  <si>
-    <t>6. Гастрономия</t>
-  </si>
-  <si>
-    <t>Приветственный ужин на вилле + тропические фрукты ежедневно (мангостины, маракуйя)</t>
-  </si>
-  <si>
-    <t>Ежедневная свежая экзотика</t>
-  </si>
-  <si>
-    <t>Авторский дегустационный сет от шефа (Mozaic / Locavore NXT)</t>
-  </si>
-  <si>
-    <t>Гастрономический флагман Азии</t>
-  </si>
-  <si>
-    <t>Панорамный закатный ужин морепродуктов на утесах Улувату</t>
-  </si>
-  <si>
-    <t>Океанский вид и свежий улов</t>
-  </si>
-  <si>
-    <t>ИТОГО ПИТАНИЕ И НАПИТКИ</t>
-  </si>
-  <si>
-    <t>Отобранные шеф-локации</t>
-  </si>
-  <si>
-    <t>7. Проводник &amp; Арт</t>
-  </si>
-  <si>
-    <t>Звукотерапия тибетскими чашами от Валерия на вилле (2 сессии)</t>
-  </si>
-  <si>
-    <t>2 сессии</t>
-  </si>
-  <si>
-    <t>Включено</t>
-  </si>
-  <si>
-    <t>Авторская практика мастера</t>
-  </si>
-  <si>
-    <t>Алхимическая портретная фотосъемка на утесах Улувату</t>
-  </si>
-  <si>
-    <t>1 сессия</t>
-  </si>
-  <si>
-    <t>Fine-art фотосессия для гостий</t>
-  </si>
-  <si>
-    <t>Интеллектуальный салон: встреча с д-ром Лоуренсом Блэром («Ring of Fire»)</t>
-  </si>
-  <si>
-    <t>1 встреча</t>
-  </si>
-  <si>
-    <t>Эксклюзивный доступ автора (35 лет экспедиций)</t>
-  </si>
-  <si>
-    <t>Частный визит в резиденцию Брюса Карпентера (сакральные крисы и маски)</t>
-  </si>
-  <si>
-    <t>1 визит</t>
-  </si>
-  <si>
-    <t>Эксперт Christie's / автор монографий</t>
-  </si>
-  <si>
-    <t>Арт-маршрут Убуда: музей Бланко, Neka Art Museum (павильон крисов), ARMA</t>
-  </si>
-  <si>
-    <t>1 день</t>
-  </si>
-  <si>
-    <t>Билеты включены в общую сакральную программу</t>
-  </si>
-  <si>
-    <t>Непрерывное кураторство 24/7 (индонезийский и английский языки)</t>
-  </si>
-  <si>
-    <t>Личное ведение без посредников</t>
-  </si>
-  <si>
-    <t>ИТОГО ОПЕРАЦИОННАЯ СЕБЕСТОИМОСТЬ (40%)</t>
-  </si>
-  <si>
-    <t>Прямые расходы на 2 гостей (отели 4★+, авто, спа, храмы, еда, VIP)</t>
-  </si>
-  <si>
-    <t>-2 388 € (чистая экономия)</t>
-  </si>
-  <si>
-    <t>40% от общей суммы пакета</t>
-  </si>
-  <si>
-    <t>ГОНОРАР МАСТЕРА ВАЛЕРИЯ ЛАТЫПОВА (60%)</t>
-  </si>
-  <si>
-    <t>Чистый гонорар за организацию, режиссуру тура и личное ведение</t>
-  </si>
-  <si>
-    <t>+4 688 € (рост гонорара)</t>
-  </si>
-  <si>
-    <t>60% чистая маржа автора</t>
-  </si>
-  <si>
-    <t>ИТОГОВАЯ СТОИМОСТЬ ПАКЕТА (ДЛЯ 2 ГОСТЕЙ)</t>
-  </si>
-  <si>
-    <t>Полный пакет «под ключ» (без международных авиабилетов)</t>
-  </si>
-  <si>
-    <t>+2 300 € (премиум Швейцария)</t>
-  </si>
-  <si>
-    <t>12 000 € за тур на двоих</t>
-  </si>
-  <si>
-    <t>СМЕТА ТУРА «BALI SANCTUARY»: 5 ДНЕЙ / 4 НОЧИ (ГОСТЬИ ИЗ ШВЕЙЦАРИИ)</t>
-  </si>
-  <si>
-    <t>Камерные бутик-отели 4★+ (300–400 €/ночь) • Полный VIP Fast-Track • Гонорар мастера 60%</t>
-  </si>
-  <si>
-    <t>Базовый расчет 5★ [€]</t>
-  </si>
-  <si>
     <t>Структура расходов</t>
   </si>
   <si>
@@ -390,13 +393,13 @@
     <t>plataran.com/plataran-ubud (320 €/н)</t>
   </si>
   <si>
-    <t>Renaissance Bali Uluwatu Resort (Ocean View Suite)</t>
+    <t>Приватная вилла у океана (Paradise Beach / Санур, 1-я линия)</t>
   </si>
   <si>
     <t>20.0% от бюджета</t>
   </si>
   <si>
-    <t>marriott.com (340 €/н)</t>
+    <t>Бутик-вилла у лагуны (340 €/н)</t>
   </si>
   <si>
     <t>Итого проживание (4 ночи, в пределах 300–400 €/ночь)</t>
@@ -522,13 +525,13 @@
     <t>Mozaic / Locavore NXT</t>
   </si>
   <si>
-    <t>Закатный панорамный ужин на скалах Улувату</t>
+    <t>Закатный праздничный ужин морепродуктов у океана (Санур)</t>
   </si>
   <si>
     <t>Морепродукты</t>
   </si>
   <si>
-    <t>Свежий улов и закат</t>
+    <t>Свежий улов и закат у воды</t>
   </si>
   <si>
     <t>Итого питание и напитки</t>
@@ -765,10 +768,10 @@
     <t>Выбрать премиум-шатер с индивидуальной геотермальной минеральной ванной на террасе. Заказать растопку купели к моменту заезда (17:00).</t>
   </si>
   <si>
-    <t>8. Отель Renaissance Uluwatu 4★+</t>
-  </si>
-  <si>
-    <t>https://www.marriott.com</t>
+    <t>8. Приватная вилла у пляжа (Санур)</t>
+  </si>
+  <si>
+    <t>Прямой контракт / Букинг виллы</t>
   </si>
   <si>
     <t>Имена гостей, даты проживания (2 ночи)</t>
@@ -777,13 +780,13 @@
     <t>5 800 000 IDR/ночь (~340 €/н)</t>
   </si>
   <si>
-    <t>Картой на официальном сайте Marriott</t>
-  </si>
-  <si>
-    <t>Подтверждение Ocean View Suite</t>
-  </si>
-  <si>
-    <t>Забронировать люкс с панорамным видом на Индийский океан. Запросить высокий этаж и поздний выезд (Late Check-out) при необходимости.</t>
+    <t>Предоплата картой или банковский перевод</t>
+  </si>
+  <si>
+    <t>Подтверждение приватной пляжной виллы</t>
+  </si>
+  <si>
+    <t>Забронировать виллу на первой линии с приватным садом и прямым выходом к спокойной лагуне для купания без волн.</t>
   </si>
   <si>
     <t>9. Ресторан Mozaic Gastronomic (Убуд)</t>
@@ -1008,10 +1011,10 @@
     <t>Вулканические горячие источники 38-40°C</t>
   </si>
   <si>
-    <t>Отель Renaissance Uluwatu 4★+</t>
-  </si>
-  <si>
-    <t>Marriott International</t>
+    <t>Приватная вилла у пляжа (Санур)</t>
+  </si>
+  <si>
+    <t>Бутик-коллекция Sanur Beachfront</t>
   </si>
   <si>
     <t>5 800 000 IDR/ночь</t>
@@ -1020,13 +1023,16 @@
     <t>340 €/ночь</t>
   </si>
   <si>
-    <t>Ocean View Suite на утесе + завтраки</t>
-  </si>
-  <si>
-    <t>Marriott Bonvoy / Прямой сайт</t>
-  </si>
-  <si>
-    <t>Панорамный бассейн над океаном</t>
+    <t>Бутик-вилла у кромки воды</t>
+  </si>
+  <si>
+    <t>Вилла с садом у лагуны + завтраки от шефа</t>
+  </si>
+  <si>
+    <t>Прямой контракт / Депозит</t>
+  </si>
+  <si>
+    <t>Тихий океан без волн, 20 мин до аэропорта DPS</t>
   </si>
   <si>
     <t>Храм Пура Бесаких</t>
@@ -2715,10 +2721,10 @@
         <v>6</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>7</v>
+        <v>120</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H4" t="s" s="1">
         <v>9</v>
@@ -2726,10 +2732,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>20</v>
@@ -2744,18 +2750,18 @@
         <v>11000000</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>20</v>
@@ -2770,21 +2776,21 @@
         <v>11600000</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="5">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B7" t="s" s="5">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s" s="5">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D7" s="5">
         <v>3700</v>
@@ -2796,10 +2802,10 @@
         <v>22600000</v>
       </c>
       <c r="G7" t="s" s="5">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H7" t="s" s="5">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8">
@@ -2807,10 +2813,10 @@
         <v>27</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D8" s="0">
         <v>400</v>
@@ -2822,10 +2828,10 @@
         <v>5500000</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9">
@@ -2833,10 +2839,10 @@
         <v>27</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D9" s="0">
         <v>100</v>
@@ -2848,10 +2854,10 @@
         <v>1800000</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10">
@@ -2859,10 +2865,10 @@
         <v>27</v>
       </c>
       <c r="B10" t="s" s="5">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s" s="5">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D10" s="5">
         <v>500</v>
@@ -2874,7 +2880,7 @@
         <v>7300000</v>
       </c>
       <c r="G10" t="s" s="5">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H10" t="s" s="5">
         <v>37</v>
@@ -2885,7 +2891,7 @@
         <v>38</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C11" t="s" s="0">
         <v>40</v>
@@ -2900,10 +2906,10 @@
         <v>2700000</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12">
@@ -2926,7 +2932,7 @@
         <v>1000000</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H12" t="s" s="0">
         <v>45</v>
@@ -2952,7 +2958,7 @@
         <v>300000</v>
       </c>
       <c r="G13" t="s" s="0">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H13" t="s" s="0">
         <v>48</v>
@@ -2963,7 +2969,7 @@
         <v>38</v>
       </c>
       <c r="B14" t="s" s="5">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C14" t="s" s="5">
         <v>40</v>
@@ -2978,7 +2984,7 @@
         <v>4000000</v>
       </c>
       <c r="G14" t="s" s="5">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H14" t="s" s="5">
         <v>51</v>
@@ -2986,10 +2992,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C15" t="s" s="0">
         <v>40</v>
@@ -3004,7 +3010,7 @@
         <v>3200000</v>
       </c>
       <c r="G15" t="s" s="0">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H15" t="s" s="0">
         <v>55</v>
@@ -3012,10 +3018,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C16" t="s" s="0">
         <v>40</v>
@@ -3030,7 +3036,7 @@
         <v>1700000</v>
       </c>
       <c r="G16" t="s" s="0">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H16" t="s" s="0">
         <v>59</v>
@@ -3038,10 +3044,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="5">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s" s="5">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C17" t="s" s="5">
         <v>61</v>
@@ -3056,7 +3062,7 @@
         <v>4900000</v>
       </c>
       <c r="G17" t="s" s="5">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H17" t="s" s="5">
         <v>63</v>
@@ -3067,7 +3073,7 @@
         <v>64</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s" s="0">
         <v>40</v>
@@ -3082,7 +3088,7 @@
         <v>1800000</v>
       </c>
       <c r="G18" t="s" s="0">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H18" t="s" s="0">
         <v>67</v>
@@ -3093,7 +3099,7 @@
         <v>64</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C19" t="s" s="0">
         <v>40</v>
@@ -3108,10 +3114,10 @@
         <v>850000</v>
       </c>
       <c r="G19" t="s" s="0">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H19" t="s" s="0">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="20">
@@ -3119,7 +3125,7 @@
         <v>64</v>
       </c>
       <c r="B20" t="s" s="5">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C20" t="s" s="5">
         <v>61</v>
@@ -3134,10 +3140,10 @@
         <v>2650000</v>
       </c>
       <c r="G20" t="s" s="5">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H20" t="s" s="5">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21">
@@ -3145,10 +3151,10 @@
         <v>77</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D21" s="0">
         <v>150</v>
@@ -3160,10 +3166,10 @@
         <v>2550000</v>
       </c>
       <c r="G21" t="s" s="0">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H21" t="s" s="0">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22">
@@ -3171,7 +3177,7 @@
         <v>77</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C22" t="s" s="0">
         <v>40</v>
@@ -3186,10 +3192,10 @@
         <v>4250000</v>
       </c>
       <c r="G22" t="s" s="0">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H22" t="s" s="0">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23">
@@ -3197,7 +3203,7 @@
         <v>77</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C23" t="s" s="0">
         <v>40</v>
@@ -3212,10 +3218,10 @@
         <v>3400000</v>
       </c>
       <c r="G23" t="s" s="0">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H23" t="s" s="0">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24">
@@ -3223,7 +3229,7 @@
         <v>77</v>
       </c>
       <c r="B24" t="s" s="5">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C24" t="s" s="5">
         <v>61</v>
@@ -3238,7 +3244,7 @@
         <v>10200000</v>
       </c>
       <c r="G24" t="s" s="5">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H24" t="s" s="5">
         <v>85</v>
@@ -3249,7 +3255,7 @@
         <v>86</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C25" t="s" s="0">
         <v>92</v>
@@ -3353,10 +3359,10 @@
         <v>86</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D29" s="0">
         <v>0</v>
@@ -3389,10 +3395,10 @@
         <v>105</v>
       </c>
       <c r="B31" t="s" s="3">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C31" t="s" s="3">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D31" s="3">
         <v>5398</v>
@@ -3404,7 +3410,7 @@
         <v>57950000</v>
       </c>
       <c r="G31" t="s" s="3">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H31" t="s" s="3">
         <v>108</v>
@@ -3418,7 +3424,7 @@
         <v>110</v>
       </c>
       <c r="C32" t="s" s="7">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D32" s="7">
         <v>2102</v>
@@ -3430,7 +3436,7 @@
         <v>86925000</v>
       </c>
       <c r="G32" t="s" s="7">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H32" t="s" s="7">
         <v>112</v>
@@ -3444,7 +3450,7 @@
         <v>114</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D33" s="2">
         <v>7500</v>
@@ -3456,10 +3462,10 @@
         <v>144875000</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H33" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3471,7 +3477,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3483,7 +3489,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="8">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -3505,288 +3511,288 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B4" t="s" s="1">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C4" t="s" s="1">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G13" t="s" s="0">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H13" t="s" s="0">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G14" t="s" s="0">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H14" t="s" s="0">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -3798,7 +3804,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3810,7 +3816,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="4">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -3832,522 +3838,522 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B4" t="s" s="1">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C4" t="s" s="1">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>47</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>248</v>
+        <v>333</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G13" t="s" s="0">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H13" t="s" s="0">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="G14" t="s" s="0">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="H14" t="s" s="0">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="G15" t="s" s="0">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="H15" t="s" s="0">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G16" t="s" s="0">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="H16" t="s" s="0">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="G17" t="s" s="0">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="H17" t="s" s="0">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="G18" t="s" s="0">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="H18" t="s" s="0">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="G19" t="s" s="0">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="H19" t="s" s="0">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
+        <v>386</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>387</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>297</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>388</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>389</v>
+      </c>
+      <c r="G20" t="s" s="0">
         <v>384</v>
       </c>
-      <c r="B20" t="s" s="0">
-        <v>385</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>296</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>297</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>386</v>
-      </c>
-      <c r="F20" t="s" s="0">
-        <v>387</v>
-      </c>
-      <c r="G20" t="s" s="0">
-        <v>382</v>
-      </c>
       <c r="H20" t="s" s="0">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G21" t="s" s="0">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="H21" t="s" s="0">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G22" t="s" s="0">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="H22" t="s" s="0">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>406</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>399</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>400</v>
+      </c>
+      <c r="F23" t="s" s="0">
+        <v>407</v>
+      </c>
+      <c r="G23" t="s" s="0">
         <v>402</v>
       </c>
-      <c r="B23" t="s" s="0">
-        <v>403</v>
-      </c>
-      <c r="C23" t="s" s="0">
-        <v>404</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>397</v>
-      </c>
-      <c r="E23" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="F23" t="s" s="0">
-        <v>405</v>
-      </c>
-      <c r="G23" t="s" s="0">
-        <v>400</v>
-      </c>
       <c r="H23" t="s" s="0">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -4359,7 +4365,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="2">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4371,7 +4377,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="8">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -4399,33 +4405,33 @@
         <v>3</v>
       </c>
       <c r="C4" t="s" s="1">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>7</v>
+        <v>120</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D5" s="0">
         <v>1050</v>
@@ -4437,21 +4443,21 @@
         <v>17850000</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D6" s="0">
         <v>1150</v>
@@ -4463,21 +4469,21 @@
         <v>19550000</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="9">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B7" t="s" s="9">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C7" t="s" s="9">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D7" s="9">
         <v>1100</v>
@@ -4489,21 +4495,21 @@
         <v>18700000</v>
       </c>
       <c r="G7" t="s" s="9">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="H7" t="s" s="9">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="5">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B8" t="s" s="5">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C8" t="s" s="5">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D8" s="5">
         <v>1050</v>
@@ -4515,21 +4521,21 @@
         <v>17850000</v>
       </c>
       <c r="G8" t="s" s="5">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="H8" t="s" s="5">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D9" s="0">
         <v>90</v>
@@ -4541,21 +4547,21 @@
         <v>1500000</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D10" s="0">
         <v>64</v>
@@ -4567,21 +4573,21 @@
         <v>1000000</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D11" s="0">
         <v>9</v>
@@ -4593,21 +4599,21 @@
         <v>150000</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="5">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B12" t="s" s="5">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C12" t="s" s="5">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D12" s="5">
         <v>99</v>
@@ -4619,21 +4625,21 @@
         <v>1650000</v>
       </c>
       <c r="G12" t="s" s="5">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="H12" t="s" s="5">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="D13" s="0">
         <v>470</v>
@@ -4645,21 +4651,21 @@
         <v>8000000</v>
       </c>
       <c r="G13" t="s" s="0">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H13" t="s" s="0">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D14" s="0">
         <v>470</v>
@@ -4671,21 +4677,21 @@
         <v>8000000</v>
       </c>
       <c r="G14" t="s" s="0">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H14" t="s" s="0">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="5">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B15" t="s" s="5">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C15" t="s" s="5">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D15" s="5">
         <v>940</v>
@@ -4697,21 +4703,21 @@
         <v>16000000</v>
       </c>
       <c r="G15" t="s" s="5">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="H15" t="s" s="5">
-        <v>453</v>
+        <v>455</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D16" s="0">
         <v>190</v>
@@ -4723,21 +4729,21 @@
         <v>3200000</v>
       </c>
       <c r="G16" t="s" s="0">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="H16" t="s" s="0">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D17" s="0">
         <v>35</v>
@@ -4749,21 +4755,21 @@
         <v>600000</v>
       </c>
       <c r="G17" t="s" s="0">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="H17" t="s" s="0">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="5">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B18" t="s" s="5">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C18" t="s" s="5">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D18" s="5">
         <v>225</v>
@@ -4775,21 +4781,21 @@
         <v>3800000</v>
       </c>
       <c r="G18" t="s" s="5">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="H18" t="s" s="5">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D19" s="0">
         <v>1060</v>
@@ -4801,21 +4807,21 @@
         <v>18000000</v>
       </c>
       <c r="G19" t="s" s="0">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="H19" t="s" s="0">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D20" s="0">
         <v>70</v>
@@ -4827,21 +4833,21 @@
         <v>1200000</v>
       </c>
       <c r="G20" t="s" s="0">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="H20" t="s" s="0">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="5">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B21" t="s" s="5">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C21" t="s" s="5">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D21" s="5">
         <v>1130</v>
@@ -4853,21 +4859,21 @@
         <v>19200000</v>
       </c>
       <c r="G21" t="s" s="5">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="H21" t="s" s="5">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D22" s="0">
         <v>35</v>
@@ -4879,21 +4885,21 @@
         <v>600000</v>
       </c>
       <c r="G22" t="s" s="0">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="H22" t="s" s="0">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="D23" s="0">
         <v>140</v>
@@ -4905,21 +4911,21 @@
         <v>2400000</v>
       </c>
       <c r="G23" t="s" s="0">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="H23" t="s" s="0">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="5">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B24" t="s" s="5">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C24" t="s" s="5">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D24" s="5">
         <v>175</v>
@@ -4931,10 +4937,10 @@
         <v>3000000</v>
       </c>
       <c r="G24" t="s" s="5">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="H24" t="s" s="5">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="25">
@@ -4949,13 +4955,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="7">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B26" t="s" s="7">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="C26" t="s" s="7">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D26" s="7">
         <v>3619</v>
@@ -4967,21 +4973,21 @@
         <v>61500000</v>
       </c>
       <c r="G26" t="s" s="7">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="H26" t="s" s="7">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="7">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B27" t="s" s="7">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C27" t="s" s="7">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D27" s="7">
         <v>6369</v>
@@ -4993,10 +4999,10 @@
         <v>108250000</v>
       </c>
       <c r="G27" t="s" s="7">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="H27" t="s" s="7">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
   </sheetData>
@@ -5008,7 +5014,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5020,7 +5026,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="8">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -5042,33 +5048,33 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B4" t="s" s="1">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C4" t="s" s="1">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B5" s="0">
         <v>105</v>
@@ -5083,18 +5089,18 @@
         <v>530000</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B6" s="0">
         <v>25</v>
@@ -5109,18 +5115,18 @@
         <v>200000</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B7" s="0">
         <v>165</v>
@@ -5135,18 +5141,18 @@
         <v>3600000</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B8" s="0">
         <v>55</v>
@@ -5161,18 +5167,18 @@
         <v>950000</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B9" s="0">
         <v>70</v>
@@ -5187,18 +5193,18 @@
         <v>1600000</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B10" s="0">
         <v>40</v>
@@ -5213,13 +5219,13 @@
         <v>700000</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="11">
@@ -5234,7 +5240,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="7">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B12" s="7">
         <v>460</v>
@@ -5249,13 +5255,13 @@
         <v>7580000</v>
       </c>
       <c r="F12" t="s" s="7">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G12" t="s" s="7">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="H12" t="s" s="7">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="13">
@@ -5270,7 +5276,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -5282,7 +5288,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="4">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -5294,7 +5300,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="4">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -5306,7 +5312,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="4">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -5318,7 +5324,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="4">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -5330,7 +5336,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="4">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>

</xml_diff>